<commit_message>
v1.7 — register integrity, byte-reproducible workbook
The parameter workbook generator emits byte-reproducible output, and
check_release.py rebuilds and compares sha256, set-compares finding/test
IDs against the documents, and emits a warn-only inspection queue of
register values not found verbatim in their cited sections (15 rows on
first run). Doc 40 → v1.8 (task closed), doc 50 → v1.7 (gate
description). No design figure changed.

Version DOI not yet reserved: the README notice still carries v1.3's
version DOI and must be updated before merge/tag (doc 50 §9).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parameter_register.xlsx
+++ b/docs/parameter_register.xlsx
@@ -6868,7 +6868,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">

</xml_diff>